<commit_message>
Build q2815 Helm hook release delivery
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R2c63cd26e7d84ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rb93fe6c2e08e42fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -322,7 +322,7 @@
         <x:v>输入获取方式</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>从交接压缩包解压到Windows11本地目录</x:v>
+        <x:v>从消息平台版本组的发版目录下载并解压到Windows11本地目录</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -399,10 +399,10 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>能力边界</x:v>
+        <x:v>岗位边界</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>Helm lint与template只证明Chart和候选清单可处理，不证明Job执行或HTTP响应发生</x:v>
+        <x:v>发布经理审阅Chart与候选清单，集群操作人员在维护窗内执行钩子并检查端点状态</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">

</xml_diff>